<commit_message>
Add SOH report for 2026-10-09
</commit_message>
<xml_diff>
--- a/reports/SOH_08_10_2026.xlsx
+++ b/reports/SOH_08_10_2026.xlsx
@@ -3835,41 +3835,45 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>9374628501294</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>API058</t>
+          <t>AWN002PROM</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>AIWINA SUPER ADULT CARE PORTABLE BAG</t>
+          <t>AIWINA Super Soft (16* 18 Pcs) 320mm 3 Pack</t>
         </is>
       </c>
       <c r="D122" s="2" t="n">
-        <v>986</v>
+        <v>0</v>
       </c>
       <c r="E122" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="F122" t="inlineStr"/>
+        <v>5000</v>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>AIWINA</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>9374628501294</t>
+          <t>8291736405123</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>AWN002PROM</t>
+          <t>AWN001PROM</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>AIWINA Super Soft (16* 18 Pcs) 320mm 3 Pack</t>
+          <t>AIWINA Super Soft (16* 24 Pcs) 245mm 3 Pack</t>
         </is>
       </c>
       <c r="D123" s="2" t="n">
@@ -3915,24 +3919,24 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>8291736405123</t>
+          <t>9305000132852</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>AWN001PROM</t>
+          <t>AWN008</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>AIWINA Super Soft (16* 24 Pcs) 245mm 3 Pack</t>
+          <t>AIWINA Super Soft (48* 6 Pcs) 330mm</t>
         </is>
       </c>
       <c r="D125" s="2" t="n">
-        <v>0</v>
+        <v>4807</v>
       </c>
       <c r="E125" s="3" t="n">
-        <v>5000</v>
+        <v>2500</v>
       </c>
       <c r="F125" t="inlineStr">
         <is>
@@ -3943,30 +3947,26 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>9305000132852</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>AWN008</t>
+          <t>API058</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>AIWINA Super Soft (48* 6 Pcs) 330mm</t>
+          <t>AIWINA SUPER ADULT CARE PORTABLE BAG</t>
         </is>
       </c>
       <c r="D126" s="2" t="n">
-        <v>4807</v>
+        <v>986</v>
       </c>
       <c r="E126" s="3" t="n">
-        <v>2500</v>
-      </c>
-      <c r="F126" t="inlineStr">
-        <is>
-          <t>AIWINA</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="F126" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -14484,24 +14484,24 @@
     <row r="506">
       <c r="A506" t="inlineStr">
         <is>
-          <t>8409730011676</t>
+          <t>9333527021878</t>
         </is>
       </c>
       <c r="B506" t="inlineStr">
         <is>
-          <t>AP0001</t>
+          <t>AP0136</t>
         </is>
       </c>
       <c r="C506" t="inlineStr">
         <is>
-          <t>COTTON FACIAL PADS PK 80</t>
+          <t>COTTON TIPS 300PK PP TUB</t>
         </is>
       </c>
       <c r="D506" s="2" t="n">
-        <v>1257</v>
+        <v>0</v>
       </c>
       <c r="E506" s="3" t="n">
-        <v>8446</v>
+        <v>7397</v>
       </c>
       <c r="F506" t="inlineStr">
         <is>
@@ -14540,24 +14540,24 @@
     <row r="508">
       <c r="A508" t="inlineStr">
         <is>
-          <t>9333527021878</t>
+          <t>8409730033906</t>
         </is>
       </c>
       <c r="B508" t="inlineStr">
         <is>
-          <t>AP0136</t>
+          <t>SW0001</t>
         </is>
       </c>
       <c r="C508" t="inlineStr">
         <is>
-          <t>COTTON TIPS 300PK PP TUB</t>
+          <t>CREPE PAPER WRAP 50.8CMx183CM</t>
         </is>
       </c>
       <c r="D508" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E508" s="3" t="n">
-        <v>7397</v>
+        <v>2922</v>
       </c>
       <c r="F508" t="inlineStr">
         <is>
@@ -14568,24 +14568,24 @@
     <row r="509">
       <c r="A509" t="inlineStr">
         <is>
-          <t>8409730033906</t>
+          <t>8409730011676</t>
         </is>
       </c>
       <c r="B509" t="inlineStr">
         <is>
-          <t>SW0001</t>
+          <t>AP0001</t>
         </is>
       </c>
       <c r="C509" t="inlineStr">
         <is>
-          <t>CREPE PAPER WRAP 50.8CMx183CM</t>
+          <t>COTTON FACIAL PADS PK 80</t>
         </is>
       </c>
       <c r="D509" s="2" t="n">
-        <v>0</v>
+        <v>1257</v>
       </c>
       <c r="E509" s="3" t="n">
-        <v>2922</v>
+        <v>8446</v>
       </c>
       <c r="F509" t="inlineStr">
         <is>
@@ -21205,24 +21205,24 @@
     <row r="746">
       <c r="A746" t="inlineStr">
         <is>
-          <t>9333527658135</t>
+          <t>9333527803795</t>
         </is>
       </c>
       <c r="B746" t="inlineStr">
         <is>
-          <t>AH4904</t>
+          <t>AH0000067</t>
         </is>
       </c>
       <c r="C746" t="inlineStr">
         <is>
-          <t>HAIR CLIP 10 PACK BLACK</t>
+          <t>HAIR CLIP 2 PIECE SET 3 ASSORTED</t>
         </is>
       </c>
       <c r="D746" s="2" t="n">
-        <v>251</v>
+        <v>0</v>
       </c>
       <c r="E746" s="3" t="n">
-        <v>5157</v>
+        <v>7713</v>
       </c>
       <c r="F746" t="inlineStr">
         <is>
@@ -21233,24 +21233,24 @@
     <row r="747">
       <c r="A747" t="inlineStr">
         <is>
-          <t>9333527803795</t>
+          <t>9333527731500</t>
         </is>
       </c>
       <c r="B747" t="inlineStr">
         <is>
-          <t>AH0000067</t>
+          <t>AH5323</t>
         </is>
       </c>
       <c r="C747" t="inlineStr">
         <is>
-          <t>HAIR CLIP 2 PIECE SET 3 ASSORTED</t>
+          <t>HAIR CLIP MODERN 4 PACK 3 ASSORTED COLORS</t>
         </is>
       </c>
       <c r="D747" s="2" t="n">
-        <v>0</v>
+        <v>861</v>
       </c>
       <c r="E747" s="3" t="n">
-        <v>7713</v>
+        <v>3923</v>
       </c>
       <c r="F747" t="inlineStr">
         <is>
@@ -21317,24 +21317,24 @@
     <row r="750">
       <c r="A750" t="inlineStr">
         <is>
-          <t>9333527731500</t>
+          <t>9333527658135</t>
         </is>
       </c>
       <c r="B750" t="inlineStr">
         <is>
-          <t>AH5323</t>
+          <t>AH4904</t>
         </is>
       </c>
       <c r="C750" t="inlineStr">
         <is>
-          <t>HAIR CLIP MODERN 4 PACK 3 ASSORTED COLORS</t>
+          <t>HAIR CLIP 10 PACK BLACK</t>
         </is>
       </c>
       <c r="D750" s="2" t="n">
-        <v>861</v>
+        <v>251</v>
       </c>
       <c r="E750" s="3" t="n">
-        <v>3923</v>
+        <v>5157</v>
       </c>
       <c r="F750" t="inlineStr">
         <is>
@@ -24990,24 +24990,24 @@
     <row r="881">
       <c r="A881" t="inlineStr">
         <is>
-          <t>4894158134009</t>
+          <t>4894158133989</t>
         </is>
       </c>
       <c r="B881" t="inlineStr">
         <is>
-          <t>XM5099</t>
+          <t>XM5097</t>
         </is>
       </c>
       <c r="C881" t="inlineStr">
         <is>
-          <t>LED BIRCH TREE 90cm WARM WHITE</t>
+          <t>LED BIRCH TREE 180cm DUAL COLOUR</t>
         </is>
       </c>
       <c r="D881" s="2" t="n">
         <v>3</v>
       </c>
       <c r="E881" s="3" t="n">
-        <v>140719</v>
+        <v>269664</v>
       </c>
       <c r="F881" t="inlineStr">
         <is>
@@ -25018,24 +25018,24 @@
     <row r="882">
       <c r="A882" t="inlineStr">
         <is>
-          <t>4894158064566</t>
+          <t>4894158145043</t>
         </is>
       </c>
       <c r="B882" t="inlineStr">
         <is>
-          <t>XM1714</t>
+          <t>XM6035</t>
         </is>
       </c>
       <c r="C882" t="inlineStr">
         <is>
-          <t>LED BIRCH TREE 180cm WARM WHITE</t>
+          <t>LED BIRCH TREE 180cm DUAL M-WW</t>
         </is>
       </c>
       <c r="D882" s="2" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E882" s="3" t="n">
-        <v>238229</v>
+        <v>269664</v>
       </c>
       <c r="F882" t="inlineStr">
         <is>
@@ -25046,24 +25046,24 @@
     <row r="883">
       <c r="A883" t="inlineStr">
         <is>
-          <t>4894158145043</t>
+          <t>4894158064566</t>
         </is>
       </c>
       <c r="B883" t="inlineStr">
         <is>
-          <t>XM6035</t>
+          <t>XM1714</t>
         </is>
       </c>
       <c r="C883" t="inlineStr">
         <is>
-          <t>LED BIRCH TREE 180cm DUAL M-WW</t>
+          <t>LED BIRCH TREE 180cm WARM WHITE</t>
         </is>
       </c>
       <c r="D883" s="2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E883" s="3" t="n">
-        <v>269664</v>
+        <v>238229</v>
       </c>
       <c r="F883" t="inlineStr">
         <is>
@@ -25074,24 +25074,24 @@
     <row r="884">
       <c r="A884" t="inlineStr">
         <is>
-          <t>4894158093023</t>
+          <t>4894158134009</t>
         </is>
       </c>
       <c r="B884" t="inlineStr">
         <is>
-          <t>XM2724</t>
+          <t>XM5099</t>
         </is>
       </c>
       <c r="C884" t="inlineStr">
         <is>
-          <t>LED CLUSTER LIGHTS 2000 MULTI</t>
+          <t>LED BIRCH TREE 90cm WARM WHITE</t>
         </is>
       </c>
       <c r="D884" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E884" s="3" t="n">
-        <v>368225</v>
+        <v>140719</v>
       </c>
       <c r="F884" t="inlineStr">
         <is>
@@ -25102,24 +25102,24 @@
     <row r="885">
       <c r="A885" t="inlineStr">
         <is>
-          <t>4894158133989</t>
+          <t>4894158093023</t>
         </is>
       </c>
       <c r="B885" t="inlineStr">
         <is>
-          <t>XM5097</t>
+          <t>XM2724</t>
         </is>
       </c>
       <c r="C885" t="inlineStr">
         <is>
-          <t>LED BIRCH TREE 180cm DUAL COLOUR</t>
+          <t>LED CLUSTER LIGHTS 2000 MULTI</t>
         </is>
       </c>
       <c r="D885" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="E885" s="3" t="n">
-        <v>269664</v>
+        <v>368225</v>
       </c>
       <c r="F885" t="inlineStr">
         <is>
@@ -29134,24 +29134,24 @@
     <row r="1029">
       <c r="A1029" t="inlineStr">
         <is>
-          <t>9333527773678</t>
+          <t>9333527690630</t>
         </is>
       </c>
       <c r="B1029" t="inlineStr">
         <is>
-          <t>AT0000027</t>
+          <t>AH5120</t>
         </is>
       </c>
       <c r="C1029" t="inlineStr">
         <is>
-          <t>MINI DENTAL FLOSS MINT 10M 3 PACK</t>
+          <t>MINI HAIR CLIP 6 PACK 2 ASSORTED</t>
         </is>
       </c>
       <c r="D1029" s="2" t="n">
-        <v>240</v>
+        <v>0</v>
       </c>
       <c r="E1029" s="3" t="n">
-        <v>10526</v>
+        <v>6856</v>
       </c>
       <c r="F1029" t="inlineStr">
         <is>
@@ -29162,24 +29162,24 @@
     <row r="1030">
       <c r="A1030" t="inlineStr">
         <is>
-          <t>9333527690630</t>
+          <t>9333527773678</t>
         </is>
       </c>
       <c r="B1030" t="inlineStr">
         <is>
-          <t>AH5120</t>
+          <t>AT0000027</t>
         </is>
       </c>
       <c r="C1030" t="inlineStr">
         <is>
-          <t>MINI HAIR CLIP 6 PACK 2 ASSORTED</t>
+          <t>MINI DENTAL FLOSS MINT 10M 3 PACK</t>
         </is>
       </c>
       <c r="D1030" s="2" t="n">
-        <v>0</v>
+        <v>240</v>
       </c>
       <c r="E1030" s="3" t="n">
-        <v>6856</v>
+        <v>10526</v>
       </c>
       <c r="F1030" t="inlineStr">
         <is>
@@ -30367,24 +30367,24 @@
     <row r="1073">
       <c r="A1073" t="inlineStr">
         <is>
-          <t>9333527688903</t>
+          <t>9333527687043</t>
         </is>
       </c>
       <c r="B1073" t="inlineStr">
         <is>
-          <t>SP0411</t>
+          <t>SP0406</t>
         </is>
       </c>
       <c r="C1073" t="inlineStr">
         <is>
-          <t>NOTEBOOK SPIRAL FLORAL A6 8ASS</t>
+          <t>NOTEBOOK SPIRAL 80 PAGES A6</t>
         </is>
       </c>
       <c r="D1073" s="2" t="n">
-        <v>538</v>
+        <v>1104</v>
       </c>
       <c r="E1073" s="3" t="n">
-        <v>9226</v>
+        <v>9200</v>
       </c>
       <c r="F1073" t="inlineStr">
         <is>
@@ -30395,24 +30395,24 @@
     <row r="1074">
       <c r="A1074" t="inlineStr">
         <is>
-          <t>9333527037817</t>
+          <t>9333527688897</t>
         </is>
       </c>
       <c r="B1074" t="inlineStr">
         <is>
-          <t>AG0222</t>
+          <t>SP0410</t>
         </is>
       </c>
       <c r="C1074" t="inlineStr">
         <is>
-          <t>NYLON BATH BALL 30GM 3PK TUB</t>
+          <t>NOTEBOOK SPIRAL FLORAL A5 8ASS</t>
         </is>
       </c>
       <c r="D1074" s="2" t="n">
-        <v>265</v>
+        <v>373</v>
       </c>
       <c r="E1074" s="3" t="n">
-        <v>11027</v>
+        <v>16913</v>
       </c>
       <c r="F1074" t="inlineStr">
         <is>
@@ -30423,24 +30423,24 @@
     <row r="1075">
       <c r="A1075" t="inlineStr">
         <is>
-          <t>9333527582744</t>
+          <t>9333527688903</t>
         </is>
       </c>
       <c r="B1075" t="inlineStr">
         <is>
-          <t>SG0474</t>
+          <t>SP0411</t>
         </is>
       </c>
       <c r="C1075" t="inlineStr">
         <is>
-          <t>NOVELTY ERASER 6 ASSORTED</t>
+          <t>NOTEBOOK SPIRAL FLORAL A6 8ASS</t>
         </is>
       </c>
       <c r="D1075" s="2" t="n">
-        <v>268</v>
+        <v>538</v>
       </c>
       <c r="E1075" s="3" t="n">
-        <v>7975</v>
+        <v>9226</v>
       </c>
       <c r="F1075" t="inlineStr">
         <is>
@@ -30451,24 +30451,24 @@
     <row r="1076">
       <c r="A1076" t="inlineStr">
         <is>
-          <t>9333527688897</t>
+          <t>9333527582744</t>
         </is>
       </c>
       <c r="B1076" t="inlineStr">
         <is>
-          <t>SP0410</t>
+          <t>SG0474</t>
         </is>
       </c>
       <c r="C1076" t="inlineStr">
         <is>
-          <t>NOTEBOOK SPIRAL FLORAL A5 8ASS</t>
+          <t>NOVELTY ERASER 6 ASSORTED</t>
         </is>
       </c>
       <c r="D1076" s="2" t="n">
-        <v>373</v>
+        <v>268</v>
       </c>
       <c r="E1076" s="3" t="n">
-        <v>16913</v>
+        <v>7975</v>
       </c>
       <c r="F1076" t="inlineStr">
         <is>
@@ -30479,24 +30479,24 @@
     <row r="1077">
       <c r="A1077" t="inlineStr">
         <is>
-          <t>9333527687043</t>
+          <t>9333527037817</t>
         </is>
       </c>
       <c r="B1077" t="inlineStr">
         <is>
-          <t>SP0406</t>
+          <t>AG0222</t>
         </is>
       </c>
       <c r="C1077" t="inlineStr">
         <is>
-          <t>NOTEBOOK SPIRAL 80 PAGES A6</t>
+          <t>NYLON BATH BALL 30GM 3PK TUB</t>
         </is>
       </c>
       <c r="D1077" s="2" t="n">
-        <v>1104</v>
+        <v>265</v>
       </c>
       <c r="E1077" s="3" t="n">
-        <v>9200</v>
+        <v>11027</v>
       </c>
       <c r="F1077" t="inlineStr">
         <is>
@@ -33307,24 +33307,24 @@
     <row r="1178">
       <c r="A1178" t="inlineStr">
         <is>
-          <t>9333527002174</t>
+          <t>9333527794260</t>
         </is>
       </c>
       <c r="B1178" t="inlineStr">
         <is>
-          <t>PG0009</t>
+          <t>PH0000131</t>
         </is>
       </c>
       <c r="C1178" t="inlineStr">
         <is>
-          <t>PET BRUSH 2 SIDED</t>
+          <t>PET CARRIER 47 X 30 X 28CM</t>
         </is>
       </c>
       <c r="D1178" s="2" t="n">
-        <v>189</v>
+        <v>0</v>
       </c>
       <c r="E1178" s="3" t="n">
-        <v>14554</v>
+        <v>145529</v>
       </c>
       <c r="F1178" t="inlineStr">
         <is>
@@ -33335,24 +33335,24 @@
     <row r="1179">
       <c r="A1179" t="inlineStr">
         <is>
-          <t>9333527004932</t>
+          <t>9333527614261</t>
         </is>
       </c>
       <c r="B1179" t="inlineStr">
         <is>
-          <t>PG0080</t>
+          <t>PG0821.</t>
         </is>
       </c>
       <c r="C1179" t="inlineStr">
         <is>
-          <t>PET CAR SAFETY HARNESS 4 SIZES</t>
+          <t>PET CAR SEAT BELT ADJUSTABLE</t>
         </is>
       </c>
       <c r="D1179" s="2" t="n">
-        <v>134</v>
+        <v>0</v>
       </c>
       <c r="E1179" s="3" t="n">
-        <v>21471</v>
+        <v>6356</v>
       </c>
       <c r="F1179" t="inlineStr">
         <is>
@@ -33363,24 +33363,24 @@
     <row r="1180">
       <c r="A1180" t="inlineStr">
         <is>
-          <t>9333527614261</t>
+          <t>9333527004932</t>
         </is>
       </c>
       <c r="B1180" t="inlineStr">
         <is>
-          <t>PG0821.</t>
+          <t>PG0080</t>
         </is>
       </c>
       <c r="C1180" t="inlineStr">
         <is>
-          <t>PET CAR SEAT BELT ADJUSTABLE</t>
+          <t>PET CAR SAFETY HARNESS 4 SIZES</t>
         </is>
       </c>
       <c r="D1180" s="2" t="n">
-        <v>0</v>
+        <v>134</v>
       </c>
       <c r="E1180" s="3" t="n">
-        <v>6356</v>
+        <v>21471</v>
       </c>
       <c r="F1180" t="inlineStr">
         <is>
@@ -33391,24 +33391,24 @@
     <row r="1181">
       <c r="A1181" t="inlineStr">
         <is>
-          <t>9333527794260</t>
+          <t>9333527693297</t>
         </is>
       </c>
       <c r="B1181" t="inlineStr">
         <is>
-          <t>PH0000131</t>
+          <t>PH4098</t>
         </is>
       </c>
       <c r="C1181" t="inlineStr">
         <is>
-          <t>PET CARRIER 47 X 30 X 28CM</t>
+          <t>PET CAVE WITH PRINT 40X25CM</t>
         </is>
       </c>
       <c r="D1181" s="2" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="E1181" s="3" t="n">
-        <v>145529</v>
+        <v>88267</v>
       </c>
       <c r="F1181" t="inlineStr">
         <is>
@@ -33419,24 +33419,24 @@
     <row r="1182">
       <c r="A1182" t="inlineStr">
         <is>
-          <t>9333527693297</t>
+          <t>9333527002174</t>
         </is>
       </c>
       <c r="B1182" t="inlineStr">
         <is>
-          <t>PH4098</t>
+          <t>PG0009</t>
         </is>
       </c>
       <c r="C1182" t="inlineStr">
         <is>
-          <t>PET CAVE WITH PRINT 40X25CM</t>
+          <t>PET BRUSH 2 SIDED</t>
         </is>
       </c>
       <c r="D1182" s="2" t="n">
-        <v>7</v>
+        <v>189</v>
       </c>
       <c r="E1182" s="3" t="n">
-        <v>88267</v>
+        <v>14554</v>
       </c>
       <c r="F1182" t="inlineStr">
         <is>

</xml_diff>